<commit_message>
Spiral 1: AKE_DEMO setup and daily tracker
</commit_message>
<xml_diff>
--- a/AKE_Project_Tracking_System_Tracker_V1.xlsx
+++ b/AKE_Project_Tracking_System_Tracker_V1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\AKE-Database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1823370-98D2-4772-A0D6-F25169231EDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{602621FD-1DC4-4A5D-8C75-045B5A58950B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="409" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="452" uniqueCount="224">
   <si>
     <t>AKE Project Tracking System</t>
   </si>
@@ -174,7 +174,13 @@
     <t>A4. SAP Environment</t>
   </si>
   <si>
-    <t>Confirmed: SAP Business One 10, SAP HANA, India localization, INR, TRAINING database (not production). NOT YET confirmed: exact B1 10 Feature Pack / patch level of the target server, server name and who creates the company DB.</t>
+    <t>SAP Business One 10.0 for SAP HANA, version 10.00.310, FP 2511 (64-bit), India localization, INR - confirmed from 'About SAP Business One' screenshot (Screenshot (1).png). Client host SSO-WINDOWS1. OPEN POINT: the About box shows the licence is issued to 'Bangalore Biotech Labs Private Limited', not AKE or Qltc - Qltc to confirm this is the right server and that the licence permits an AKE training company.</t>
+  </si>
+  <si>
+    <t>Screenshot (1).png</t>
+  </si>
+  <si>
+    <t>Target build: B1 10.0 FP 2511 (10.00.310) on HANA. All DTW templates, Service Layer payloads and SQL checks built for this version.</t>
   </si>
   <si>
     <t>A5. Selling Price Confidentiality</t>
@@ -186,10 +192,16 @@
     <t>DRAFT: Trainees must be able to run OTC end-to-end without ever seeing a real selling price. Success = no real price visible in price lists, item master, sales documents, gross profit window or reports under any trainee login.</t>
   </si>
   <si>
-    <t>DRAFT options: (1) dummy prices only in the training DB; (2) authorizations - Price Lists = No Authorization, Gross Profit = No Authorization, Item Master price tab hidden; (3) both. Recommended: both.</t>
-  </si>
-  <si>
-    <t>Risk: authorizations alone can leak via reports/Excel export - dummy prices remove the risk at source.</t>
+    <t>Chosen: both layers - only dummy sales prices exist in the DB ('Sales Price (Dummy - Restricted)' price list, FG items only) + No Authorization on Price Lists, Gross Profit and Sales Analysis for all users except TRAINER.</t>
+  </si>
+  <si>
+    <t>Authorizations are set manually - Service Layer cannot set general authorizations.</t>
+  </si>
+  <si>
+    <t>Built: price lists + dummy FG prices in data package; authorization settings in checklist Step 7. Awaiting load and SUNIL-login test.</t>
+  </si>
+  <si>
+    <t>tools/build_data.py -&gt; data/*.json; tools/sl_loader.py; docs/01_Company_Setup_Checklist.md</t>
   </si>
   <si>
     <t>Overall % Complete</t>
@@ -204,7 +216,16 @@
     <t>B1. Inventory Not Matching Physical Stock</t>
   </si>
   <si>
-    <t>Stated by Qltc: system inventory does not match physical inventory. NOT YET explored: which item groups/warehouses are worst, whether production issues are backflushed or manual, whether GRPOs are posted on receipt, last physical count date. Early evidence from COA: separate Stock Difference Gain/Loss and Revaluation accounts exist (4001-18 to 4001-21) but 10 inventory group accounts are blank (5002-01-01-14, -19, -21, -22, -24 to -29) and WIP exists twice (5002-01-01-15 and 5002-01-02).</t>
+    <t>Answers (Qltc, 1 Oct 2026): most item groups AND warehouses mismatch; Issue for Production is done MANUALLY; GRPO is posted when goods arrive (purchase items); Receipt from Production is posted for produced items. Supporting COA evidence: 10 blank inventory group accounts, WIP held in two accounts (5002-01-01-15 and 5002-01-02).</t>
+  </si>
+  <si>
+    <t>DRAFT: Ashok needs system stock to equal physical stock in every warehouse. With manual Issue for Production, components are issued late, partially or in wrong quantities (and with wrong BOM quantities - see B3), so stock drifts while GRPO/Receipt keep adding to it. Training must show: correct issue against a production order, warehouse-wise stock check, Inventory Counting and Posting to correct differences.</t>
+  </si>
+  <si>
+    <t>Chosen: 6 clear warehouses (RM-STR, CONS, SHOP, FG, SCRAP, SITE), manual Issue for Production kept (AKE's real practice), Block negative inventory = Yes, dummy opening stock per warehouse, Inventory Counting exercise in training.</t>
+  </si>
+  <si>
+    <t>Built: warehouses, items with manual issue method, opening stock (30 lines). Awaiting load.</t>
   </si>
   <si>
     <t>B2. Finance Reports Not Coming Properly</t>
@@ -222,7 +243,16 @@
     <t>B3. BOM Needs Correction</t>
   </si>
   <si>
-    <t>Stated by Qltc: BOMs need to be corrected. NOT YET explored: which BOMs, what is wrong (quantities, missing components, wrong BOM type, no resources/routing), and whether AKE's real BOMs can be shared. Training DB will use dummy fabrication BOMs unless samples are provided.</t>
+    <t>Answers (Qltc, 1 Oct 2026): BOM quantities do not match reality - wrong quantity entries on BOM lines. Training DB will use dummy fabrication BOMs with realistic quantities (weight-based steel: kg per unit), plus one deliberately wrong BOM to demonstrate the effect.</t>
+  </si>
+  <si>
+    <t>DRAFT: Wrong BOM quantities make every production order issue the wrong components, so stock and product cost are wrong even when users follow the process. Training must show how a wrong BOM quantity flows into Issue for Production, stock and cost - and how to correct it.</t>
+  </si>
+  <si>
+    <t>Chosen: 5 production BOMs with realistic steel weights (e.g. ISMB300 6m column = 265.2 kg) incl. resources; the 'wrong BOM' (2652 kg decimal slip) is a live trainer exercise, not loaded.</t>
+  </si>
+  <si>
+    <t>Built: 09_boms.json (2 sub-assemblies, 3 FG). Awaiting load.</t>
   </si>
   <si>
     <t>B4. Users Not Aware of SAP B1</t>
@@ -240,7 +270,16 @@
     <t>Decision (Qltc, 1 Oct 2026): use AKE's real Chart of Accounts, not the standard India template, and use it to show AKE the finance report problems. Export received as 5 files (Asset 199, Liability 122, Equity 12, Revenue 37, Expenditure 228 accounts) and pushed to GitHub.</t>
   </si>
   <si>
-    <t>DRAFT: Load AKE's COA so trainees recognise their own accounts, but the training DB must also demonstrate the corrected structure. Open decision: load AS-IS (to show the problem) and correct live in the Finance session, or load a corrected copy plus a before/after report.</t>
+    <t>Decision (Qltc, 1 Oct 2026): load AKE's Chart of Accounts EXACTLY as given (as-is, all 598 accounts), so trainees see their own structure and the COA Findings can be demonstrated live in the Finance session. Corrections are shown, not pre-applied.</t>
+  </si>
+  <si>
+    <t>Chosen: load 598 accounts as given. Parents rebuilt from codes + file order (export lost indentation); 42 placed by position; 36 blank names get placeholder '(No name in AKE COA) &lt;code&gt;' because B1 requires a name.</t>
+  </si>
+  <si>
+    <t>Placement of 42 accounts is reconstructed - verify against OACT (FatherNum, Levels) from AKE's SQL DB if exact tree matters.</t>
+  </si>
+  <si>
+    <t>Built: 01_chart_of_accounts.json + 01_coa_placement_review.json. Dry-run OK (598 posts). Awaiting load.</t>
   </si>
   <si>
     <t>C2. Tax - GST and TDS (No e-Invoice)</t>
@@ -249,22 +288,55 @@
     <t>Decision (Qltc, 1 Oct 2026): GST + TDS required; e-Invoice out of scope. Note: TDS is not written in the design document - recorded here as Qltc's instruction. AKE already uses TDS @0.75%, 1%, 1.5%, 2%, 7.5%, 10%, on Rent, Professional, Purchases (194Q) and Interest.</t>
   </si>
   <si>
+    <t>Chosen: 4 GST codes (CGST+SGST / IGST at 18% and 12%) and 6 TDS codes (194Q, 194C1, 194C2, 194J, 194I, 194A) on AKE's existing accounts.</t>
+  </si>
+  <si>
+    <t>India tax setup is manual - not loaded via Service Layer.</t>
+  </si>
+  <si>
+    <t>Built: 07_gst_codes.json, 07_tds_codes.json; setup in checklist Steps 5-6 (manual). HSN per item in data package.</t>
+  </si>
+  <si>
     <t>C3. Master Data - Realistic Dummy Items &amp; BPs</t>
   </si>
   <si>
     <t>Decision (Qltc, 1 Oct 2026): realistic dummy data, not AKE's live masters. Items follow AKE's own item groups (RM Plates, RM Structurals, RM Special Grades, TMT Rod, Consumables, Tools, PPE, Sub Assembly, FG). Indian vendors and customers with dummy GSTIN/PAN.</t>
   </si>
   <si>
+    <t>Chosen: 37 dummy items across AKE's 9 item groups; 9 fictional vendors + 6 fictional customers in KA/TN/MH/TS/KL with checksum-valid dummy GSTIN.</t>
+  </si>
+  <si>
+    <t>Built: 05_items.json, 06_business_partners.json. Dry-run OK. Awaiting load.</t>
+  </si>
+  <si>
     <t>C4. Opening Balances &amp; Posting Periods</t>
   </si>
   <si>
-    <t>NOT YET confirmed: financial year (assume FY 2026-27, Apr-Mar), posting period granularity, and whether opening balances (stock, BP, GL) should be loaded as dummy values.</t>
+    <t>Decision (Qltc, 1 Oct 2026): use DUMMY opening balances (stock, BP, GL). Financial year assumed FY 2026-27 (Apr 2026 - Mar 2027), monthly posting periods.</t>
+  </si>
+  <si>
+    <t>Opening balances: dummy stock per item/warehouse, dummy BP balances, dummy GL balances against 1003 Opening Balance Offset Account.</t>
+  </si>
+  <si>
+    <t>Chosen: opening date 01-Apr-2026 against 1003 Opening Balance Offset Account - stock via Goods Receipt, BP and GL via Journal Entries.</t>
+  </si>
+  <si>
+    <t>Built: 11_opening_balances.json (30 stock lines, 6 BP, 10 GL). Awaiting load.</t>
   </si>
   <si>
     <t>C5. Users, Licences &amp; Authorizations</t>
   </si>
   <si>
-    <t>Known: 5 participants (+ trainer). NOT YET confirmed: number and type of licences on the training server, user codes, whether Directors get full or restricted access.</t>
+    <t>Decision (Qltc, 1 Oct 2026): 6 user licences - Rashmi, Namrata, Ashok, Sunil, Veena + trainer (manager). Licence type not yet stated (assume Professional).</t>
+  </si>
+  <si>
+    <t>6 users, role-based authorizations; selling prices hidden for all trainee users (A5).</t>
+  </si>
+  <si>
+    <t>Chosen: 6 users (TRAINER superuser), role matrix in checklist Step 7; licences assigned manually.</t>
+  </si>
+  <si>
+    <t>Built: 10_users.json; passwords from git-ignored .env. Awaiting load.</t>
   </si>
   <si>
     <t>D. Method &amp; Delivery</t>
@@ -288,7 +360,16 @@
     <t>D3. Delivery Mechanism - Access to SAP</t>
   </si>
   <si>
-    <t>Claude cannot reach the SAP server. NOT YET decided: Qltc runs the deliverables (setup checklist, DTW templates, HANA SQL checks), or Qltc provides Service Layer access to a test server so data can be posted directly.</t>
+    <t>Decision (Qltc, 1 Oct 2026): Qltc will provide Service Layer access - data will be posted directly by Claude. Credentials to be kept in a local, git-ignored file - never committed to the public repo. Pending: Service Layer URL, company DB name, user.</t>
+  </si>
+  <si>
+    <t>Loader posts all masters and opening balances through Service Layer; Qltc creates the empty company and does the manual setup steps (G/L determination, GST, TDS, licences, authorizations).</t>
+  </si>
+  <si>
+    <t>Chosen: idempotent Python loader (skips existing records, logs every call), dry-run mode, credentials only in .env.</t>
+  </si>
+  <si>
+    <t>Built and dry-run tested (all 13 steps). Not yet run against the server - expect a short fix-and-rerun loop on first contact.</t>
   </si>
   <si>
     <t>D4. Source Control</t>
@@ -580,6 +661,24 @@
   </si>
   <si>
     <t>Correct names during training-DB load.</t>
+  </si>
+  <si>
+    <t>F14</t>
+  </si>
+  <si>
+    <t>Product sales posted to an unnamed account</t>
+  </si>
+  <si>
+    <t>2001-01-01 SALES-PRODUCT SALES; 2001-01-01-01 (no name)</t>
+  </si>
+  <si>
+    <t>2001-01-01 is a title account; its only postable child 2001-01-01-01 has no name. Product sales revenue can only be posted to the unnamed account.</t>
+  </si>
+  <si>
+    <t>The main revenue line of the P&amp;L appears without a name; sales analysis by GL is unreadable.</t>
+  </si>
+  <si>
+    <t>Name 2001-01-01-01 'Sales - Product Sales (Domestic)' and use it in G/L determination.</t>
   </si>
   <si>
     <t>Summary</t>
@@ -1115,17 +1214,17 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>12</c:v>
+                  <c:v>32</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>78</c:v>
+                  <c:v>58</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-6983-45ED-9838-9733FB2559B7}"/>
+              <c16:uniqueId val="{00000000-0AA8-4C63-A5EA-C00DE9EB167F}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1240,13 +1339,13 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>12</c:v>
+                  <c:v>18</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>5</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>9</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -1259,7 +1358,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-AD56-437B-81EC-56B9E53253A5}"/>
+              <c16:uniqueId val="{00000000-728F-416F-8E8A-6EE40EAE1796}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1313,13 +1412,13 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>6</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>18</c:v>
+                  <c:v>13</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>18</c:v>
+                  <c:v>9</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>18</c:v>
@@ -1332,7 +1431,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-AD56-437B-81EC-56B9E53253A5}"/>
+              <c16:uniqueId val="{00000001-728F-416F-8E8A-6EE40EAE1796}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1813,12 +1912,12 @@
       <c r="B5" s="47"/>
       <c r="C5" s="39">
         <f>'AKE Tracking System V1'!AH7</f>
-        <v>0.13333333333333333</v>
+        <v>0.35555555555555557</v>
       </c>
       <c r="D5" s="40"/>
       <c r="E5" s="43" t="str">
         <f>INDEX($A$11:$A$15,MATCH(MIN($E$11:$E$15),$E$11:$E$15,0))</f>
-        <v>Define</v>
+        <v>Prototype</v>
       </c>
       <c r="F5" s="44"/>
       <c r="G5" s="41">
@@ -1875,11 +1974,11 @@
       </c>
       <c r="B11" s="4">
         <f>COUNTIF('AKE Tracking System V1'!B2:B200,"Closed")</f>
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="C11" s="4">
         <f>COUNTIF('AKE Tracking System V1'!B2:B200,"Open")</f>
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="D11" s="4">
         <f>B11+C11</f>
@@ -1887,7 +1986,7 @@
       </c>
       <c r="E11" s="5">
         <f>IF(D11=0,0,B11/D11)</f>
-        <v>0.66666666666666663</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:9">
@@ -1896,11 +1995,11 @@
       </c>
       <c r="B12" s="7">
         <f>COUNTIF('AKE Tracking System V1'!H2:H200,"Closed")</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="C12" s="7">
         <f>COUNTIF('AKE Tracking System V1'!H2:H200,"Open")</f>
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="D12" s="7">
         <f>B12+C12</f>
@@ -1908,7 +2007,7 @@
       </c>
       <c r="E12" s="8">
         <f>IF(D12=0,0,B12/D12)</f>
-        <v>0</v>
+        <v>0.27777777777777779</v>
       </c>
     </row>
     <row r="13" spans="1:9">
@@ -1917,11 +2016,11 @@
       </c>
       <c r="B13" s="4">
         <f>COUNTIF('AKE Tracking System V1'!N2:N200,"Closed")</f>
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="C13" s="4">
         <f>COUNTIF('AKE Tracking System V1'!N2:N200,"Open")</f>
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D13" s="4">
         <f>B13+C13</f>
@@ -1929,7 +2028,7 @@
       </c>
       <c r="E13" s="5">
         <f>IF(D13=0,0,B13/D13)</f>
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="14" spans="1:9">
@@ -1980,7 +2079,7 @@
       </c>
       <c r="B22" s="12">
         <f>SUM(B11:B15)</f>
-        <v>12</v>
+        <v>32</v>
       </c>
     </row>
     <row r="23" spans="1:2">
@@ -1989,7 +2088,7 @@
       </c>
       <c r="B23" s="12">
         <f>SUM(C11:C15)</f>
-        <v>78</v>
+        <v>58</v>
       </c>
     </row>
     <row r="42" spans="1:9">
@@ -2349,12 +2448,12 @@
         <v>46296</v>
       </c>
     </row>
-    <row r="6" spans="1:34" ht="58">
+    <row r="6" spans="1:34" ht="87">
       <c r="A6" s="21" t="s">
         <v>45</v>
       </c>
       <c r="B6" s="21" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C6" s="21" t="s">
         <v>46</v>
@@ -2365,11 +2464,20 @@
       <c r="E6" s="22">
         <v>46296</v>
       </c>
+      <c r="F6" s="21" t="s">
+        <v>47</v>
+      </c>
       <c r="H6" s="21" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I6" s="21" t="s">
-        <v>35</v>
+        <v>48</v>
+      </c>
+      <c r="J6" s="21" t="s">
+        <v>34</v>
+      </c>
+      <c r="K6" s="22">
+        <v>46296</v>
       </c>
       <c r="N6" s="21" t="s">
         <v>9</v>
@@ -2396,15 +2504,15 @@
         <v>46296</v>
       </c>
     </row>
-    <row r="7" spans="1:34" ht="58">
+    <row r="7" spans="1:34" ht="188.5">
       <c r="A7" s="21" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B7" s="21" t="s">
         <v>8</v>
       </c>
       <c r="C7" s="21" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="D7" s="21" t="s">
         <v>40</v>
@@ -2416,7 +2524,7 @@
         <v>9</v>
       </c>
       <c r="I7" s="21" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="J7" s="21" t="s">
         <v>34</v>
@@ -2425,13 +2533,13 @@
         <v>46296</v>
       </c>
       <c r="N7" s="21" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="O7" s="21" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="P7" s="21" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="Q7" s="21" t="s">
         <v>34</v>
@@ -2443,7 +2551,16 @@
         <v>9</v>
       </c>
       <c r="V7" s="21" t="s">
-        <v>35</v>
+        <v>54</v>
+      </c>
+      <c r="W7" s="21" t="s">
+        <v>34</v>
+      </c>
+      <c r="X7" s="22">
+        <v>46296</v>
+      </c>
+      <c r="Y7" s="21" t="s">
+        <v>55</v>
       </c>
       <c r="AA7" s="21" t="s">
         <v>9</v>
@@ -2452,33 +2569,33 @@
         <v>35</v>
       </c>
       <c r="AG7" s="4" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="AH7" s="23">
         <f>IF((COUNTIF(B2:B23,"Closed")+COUNTIF(B2:B23,"Open")+COUNTIF(H2:H23,"Closed")+COUNTIF(H2:H23,"Open")+COUNTIF(N2:N23,"Closed")+COUNTIF(N2:N23,"Open")+COUNTIF(U2:U23,"Closed")+COUNTIF(U2:U23,"Open")+COUNTIF(AA2:AA23,"Closed")+COUNTIF(AA2:AA23,"Open"))=0,0,(COUNTIF(B2:B23,"Closed")+COUNTIF(H2:H23,"Closed")+COUNTIF(N2:N23,"Closed")+COUNTIF(U2:U23,"Closed")+COUNTIF(AA2:AA23,"Closed"))/(COUNTIF(B2:B23,"Closed")+COUNTIF(B2:B23,"Open")+COUNTIF(H2:H23,"Closed")+COUNTIF(H2:H23,"Open")+COUNTIF(N2:N23,"Closed")+COUNTIF(N2:N23,"Open")+COUNTIF(U2:U23,"Closed")+COUNTIF(U2:U23,"Open")+COUNTIF(AA2:AA23,"Closed")+COUNTIF(AA2:AA23,"Open")))</f>
-        <v>0.13333333333333333</v>
+        <v>0.35555555555555557</v>
       </c>
     </row>
     <row r="8" spans="1:34">
       <c r="A8" s="20" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="AG8" s="4" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="AH8" s="22">
         <v>46300</v>
       </c>
     </row>
-    <row r="9" spans="1:34" ht="116">
+    <row r="9" spans="1:34" ht="188.5">
       <c r="A9" s="21" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="B9" s="21" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C9" s="21" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="D9" s="21" t="s">
         <v>34</v>
@@ -2490,19 +2607,40 @@
         <v>9</v>
       </c>
       <c r="I9" s="21" t="s">
-        <v>35</v>
+        <v>61</v>
+      </c>
+      <c r="J9" s="21" t="s">
+        <v>34</v>
+      </c>
+      <c r="K9" s="22">
+        <v>46296</v>
       </c>
       <c r="N9" s="21" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="O9" s="21" t="s">
-        <v>35</v>
+        <v>62</v>
+      </c>
+      <c r="Q9" s="21" t="s">
+        <v>34</v>
+      </c>
+      <c r="R9" s="22">
+        <v>46296</v>
       </c>
       <c r="U9" s="21" t="s">
         <v>9</v>
       </c>
       <c r="V9" s="21" t="s">
-        <v>35</v>
+        <v>63</v>
+      </c>
+      <c r="W9" s="21" t="s">
+        <v>34</v>
+      </c>
+      <c r="X9" s="22">
+        <v>46296</v>
+      </c>
+      <c r="Y9" s="21" t="s">
+        <v>55</v>
       </c>
       <c r="AA9" s="21" t="s">
         <v>9</v>
@@ -2513,13 +2651,13 @@
     </row>
     <row r="10" spans="1:34" ht="116">
       <c r="A10" s="21" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="B10" s="21" t="s">
         <v>8</v>
       </c>
       <c r="C10" s="21" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="D10" s="21" t="s">
         <v>34</v>
@@ -2528,13 +2666,13 @@
         <v>46296</v>
       </c>
       <c r="F10" s="21" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="H10" s="21" t="s">
         <v>9</v>
       </c>
       <c r="I10" s="21" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="J10" s="21" t="s">
         <v>34</v>
@@ -2561,15 +2699,15 @@
         <v>35</v>
       </c>
     </row>
-    <row r="11" spans="1:34" ht="72.5">
+    <row r="11" spans="1:34" ht="188.5">
       <c r="A11" s="21" t="s">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="B11" s="21" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C11" s="21" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="D11" s="21" t="s">
         <v>40</v>
@@ -2581,19 +2719,40 @@
         <v>9</v>
       </c>
       <c r="I11" s="21" t="s">
-        <v>35</v>
+        <v>70</v>
+      </c>
+      <c r="J11" s="21" t="s">
+        <v>34</v>
+      </c>
+      <c r="K11" s="22">
+        <v>46296</v>
       </c>
       <c r="N11" s="21" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="O11" s="21" t="s">
-        <v>35</v>
+        <v>71</v>
+      </c>
+      <c r="Q11" s="21" t="s">
+        <v>34</v>
+      </c>
+      <c r="R11" s="22">
+        <v>46296</v>
       </c>
       <c r="U11" s="21" t="s">
         <v>9</v>
       </c>
       <c r="V11" s="21" t="s">
-        <v>35</v>
+        <v>72</v>
+      </c>
+      <c r="W11" s="21" t="s">
+        <v>34</v>
+      </c>
+      <c r="X11" s="22">
+        <v>46296</v>
+      </c>
+      <c r="Y11" s="21" t="s">
+        <v>55</v>
       </c>
       <c r="AA11" s="21" t="s">
         <v>9</v>
@@ -2604,13 +2763,13 @@
     </row>
     <row r="12" spans="1:34" ht="43.5">
       <c r="A12" s="21" t="s">
-        <v>63</v>
+        <v>73</v>
       </c>
       <c r="B12" s="21" t="s">
         <v>8</v>
       </c>
       <c r="C12" s="21" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="D12" s="21" t="s">
         <v>40</v>
@@ -2645,18 +2804,18 @@
     </row>
     <row r="13" spans="1:34">
       <c r="A13" s="20" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="14" spans="1:34" ht="87">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="14" spans="1:34" ht="188.5">
       <c r="A14" s="21" t="s">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="B14" s="21" t="s">
         <v>8</v>
       </c>
       <c r="C14" s="21" t="s">
-        <v>67</v>
+        <v>77</v>
       </c>
       <c r="D14" s="21" t="s">
         <v>40</v>
@@ -2665,31 +2824,49 @@
         <v>46296</v>
       </c>
       <c r="F14" s="21" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="H14" s="21" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I14" s="21" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="J14" s="21" t="s">
+        <v>40</v>
+      </c>
+      <c r="K14" s="22">
+        <v>46296</v>
+      </c>
+      <c r="N14" s="21" t="s">
+        <v>8</v>
+      </c>
+      <c r="O14" s="21" t="s">
+        <v>79</v>
+      </c>
+      <c r="P14" s="21" t="s">
+        <v>80</v>
+      </c>
+      <c r="Q14" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="K14" s="22">
-        <v>46296</v>
-      </c>
-      <c r="N14" s="21" t="s">
-        <v>9</v>
-      </c>
-      <c r="O14" s="21" t="s">
-        <v>35</v>
+      <c r="R14" s="22">
+        <v>46296</v>
       </c>
       <c r="U14" s="21" t="s">
         <v>9</v>
       </c>
       <c r="V14" s="21" t="s">
-        <v>35</v>
+        <v>81</v>
+      </c>
+      <c r="W14" s="21" t="s">
+        <v>34</v>
+      </c>
+      <c r="X14" s="22">
+        <v>46296</v>
+      </c>
+      <c r="Y14" s="21" t="s">
+        <v>55</v>
       </c>
       <c r="AA14" s="21" t="s">
         <v>9</v>
@@ -2698,15 +2875,15 @@
         <v>35</v>
       </c>
     </row>
-    <row r="15" spans="1:34" ht="58">
+    <row r="15" spans="1:34" ht="188.5">
       <c r="A15" s="21" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="B15" s="21" t="s">
         <v>8</v>
       </c>
       <c r="C15" s="21" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="D15" s="21" t="s">
         <v>40</v>
@@ -2721,16 +2898,34 @@
         <v>35</v>
       </c>
       <c r="N15" s="21" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="O15" s="21" t="s">
-        <v>35</v>
+        <v>84</v>
+      </c>
+      <c r="P15" s="21" t="s">
+        <v>85</v>
+      </c>
+      <c r="Q15" s="21" t="s">
+        <v>34</v>
+      </c>
+      <c r="R15" s="22">
+        <v>46296</v>
       </c>
       <c r="U15" s="21" t="s">
         <v>9</v>
       </c>
       <c r="V15" s="21" t="s">
-        <v>35</v>
+        <v>86</v>
+      </c>
+      <c r="W15" s="21" t="s">
+        <v>34</v>
+      </c>
+      <c r="X15" s="22">
+        <v>46296</v>
+      </c>
+      <c r="Y15" s="21" t="s">
+        <v>55</v>
       </c>
       <c r="AA15" s="21" t="s">
         <v>9</v>
@@ -2739,15 +2934,15 @@
         <v>35</v>
       </c>
     </row>
-    <row r="16" spans="1:34" ht="72.5">
+    <row r="16" spans="1:34" ht="188.5">
       <c r="A16" s="21" t="s">
-        <v>71</v>
+        <v>87</v>
       </c>
       <c r="B16" s="21" t="s">
         <v>8</v>
       </c>
       <c r="C16" s="21" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="D16" s="21" t="s">
         <v>40</v>
@@ -2762,16 +2957,31 @@
         <v>35</v>
       </c>
       <c r="N16" s="21" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="O16" s="21" t="s">
-        <v>35</v>
+        <v>89</v>
+      </c>
+      <c r="Q16" s="21" t="s">
+        <v>34</v>
+      </c>
+      <c r="R16" s="22">
+        <v>46296</v>
       </c>
       <c r="U16" s="21" t="s">
         <v>9</v>
       </c>
       <c r="V16" s="21" t="s">
-        <v>35</v>
+        <v>90</v>
+      </c>
+      <c r="W16" s="21" t="s">
+        <v>34</v>
+      </c>
+      <c r="X16" s="22">
+        <v>46296</v>
+      </c>
+      <c r="Y16" s="21" t="s">
+        <v>55</v>
       </c>
       <c r="AA16" s="21" t="s">
         <v>9</v>
@@ -2780,15 +2990,15 @@
         <v>35</v>
       </c>
     </row>
-    <row r="17" spans="1:28" ht="43.5">
+    <row r="17" spans="1:28" ht="188.5">
       <c r="A17" s="21" t="s">
-        <v>73</v>
+        <v>91</v>
       </c>
       <c r="B17" s="21" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C17" s="21" t="s">
-        <v>74</v>
+        <v>92</v>
       </c>
       <c r="D17" s="21" t="s">
         <v>40</v>
@@ -2797,22 +3007,43 @@
         <v>46296</v>
       </c>
       <c r="H17" s="21" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I17" s="21" t="s">
-        <v>35</v>
+        <v>93</v>
+      </c>
+      <c r="J17" s="21" t="s">
+        <v>34</v>
+      </c>
+      <c r="K17" s="22">
+        <v>46296</v>
       </c>
       <c r="N17" s="21" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="O17" s="21" t="s">
-        <v>35</v>
+        <v>94</v>
+      </c>
+      <c r="Q17" s="21" t="s">
+        <v>34</v>
+      </c>
+      <c r="R17" s="22">
+        <v>46296</v>
       </c>
       <c r="U17" s="21" t="s">
         <v>9</v>
       </c>
       <c r="V17" s="21" t="s">
-        <v>35</v>
+        <v>95</v>
+      </c>
+      <c r="W17" s="21" t="s">
+        <v>34</v>
+      </c>
+      <c r="X17" s="22">
+        <v>46296</v>
+      </c>
+      <c r="Y17" s="21" t="s">
+        <v>55</v>
       </c>
       <c r="AA17" s="21" t="s">
         <v>9</v>
@@ -2821,15 +3052,15 @@
         <v>35</v>
       </c>
     </row>
-    <row r="18" spans="1:28" ht="43.5">
+    <row r="18" spans="1:28" ht="188.5">
       <c r="A18" s="21" t="s">
-        <v>75</v>
+        <v>96</v>
       </c>
       <c r="B18" s="21" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C18" s="21" t="s">
-        <v>76</v>
+        <v>97</v>
       </c>
       <c r="D18" s="21" t="s">
         <v>40</v>
@@ -2838,22 +3069,43 @@
         <v>46296</v>
       </c>
       <c r="H18" s="21" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I18" s="21" t="s">
-        <v>35</v>
+        <v>98</v>
+      </c>
+      <c r="J18" s="21" t="s">
+        <v>34</v>
+      </c>
+      <c r="K18" s="22">
+        <v>46296</v>
       </c>
       <c r="N18" s="21" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="O18" s="21" t="s">
-        <v>35</v>
+        <v>99</v>
+      </c>
+      <c r="Q18" s="21" t="s">
+        <v>34</v>
+      </c>
+      <c r="R18" s="22">
+        <v>46296</v>
       </c>
       <c r="U18" s="21" t="s">
         <v>9</v>
       </c>
       <c r="V18" s="21" t="s">
-        <v>35</v>
+        <v>100</v>
+      </c>
+      <c r="W18" s="21" t="s">
+        <v>34</v>
+      </c>
+      <c r="X18" s="22">
+        <v>46296</v>
+      </c>
+      <c r="Y18" s="21" t="s">
+        <v>55</v>
       </c>
       <c r="AA18" s="21" t="s">
         <v>9</v>
@@ -2864,18 +3116,18 @@
     </row>
     <row r="19" spans="1:28">
       <c r="A19" s="20" t="s">
-        <v>77</v>
+        <v>101</v>
       </c>
     </row>
     <row r="20" spans="1:28" ht="87">
       <c r="A20" s="21" t="s">
-        <v>78</v>
+        <v>102</v>
       </c>
       <c r="B20" s="21" t="s">
         <v>8</v>
       </c>
       <c r="C20" s="21" t="s">
-        <v>79</v>
+        <v>103</v>
       </c>
       <c r="D20" s="21" t="s">
         <v>40</v>
@@ -2884,7 +3136,7 @@
         <v>46296</v>
       </c>
       <c r="F20" s="21" t="s">
-        <v>80</v>
+        <v>104</v>
       </c>
       <c r="H20" s="21" t="s">
         <v>9</v>
@@ -2913,13 +3165,13 @@
     </row>
     <row r="21" spans="1:28" ht="29">
       <c r="A21" s="21" t="s">
-        <v>81</v>
+        <v>105</v>
       </c>
       <c r="B21" s="21" t="s">
         <v>8</v>
       </c>
       <c r="C21" s="21" t="s">
-        <v>82</v>
+        <v>106</v>
       </c>
       <c r="D21" s="21" t="s">
         <v>40</v>
@@ -2952,15 +3204,15 @@
         <v>35</v>
       </c>
     </row>
-    <row r="22" spans="1:28" ht="58">
+    <row r="22" spans="1:28" ht="188.5">
       <c r="A22" s="21" t="s">
-        <v>83</v>
+        <v>107</v>
       </c>
       <c r="B22" s="21" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C22" s="21" t="s">
-        <v>84</v>
+        <v>108</v>
       </c>
       <c r="D22" s="21" t="s">
         <v>34</v>
@@ -2969,22 +3221,43 @@
         <v>46296</v>
       </c>
       <c r="H22" s="21" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I22" s="21" t="s">
-        <v>35</v>
+        <v>109</v>
+      </c>
+      <c r="J22" s="21" t="s">
+        <v>34</v>
+      </c>
+      <c r="K22" s="22">
+        <v>46296</v>
       </c>
       <c r="N22" s="21" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="O22" s="21" t="s">
-        <v>35</v>
+        <v>110</v>
+      </c>
+      <c r="Q22" s="21" t="s">
+        <v>34</v>
+      </c>
+      <c r="R22" s="22">
+        <v>46296</v>
       </c>
       <c r="U22" s="21" t="s">
         <v>9</v>
       </c>
       <c r="V22" s="21" t="s">
-        <v>35</v>
+        <v>111</v>
+      </c>
+      <c r="W22" s="21" t="s">
+        <v>34</v>
+      </c>
+      <c r="X22" s="22">
+        <v>46296</v>
+      </c>
+      <c r="Y22" s="21" t="s">
+        <v>55</v>
       </c>
       <c r="AA22" s="21" t="s">
         <v>9</v>
@@ -2995,13 +3268,13 @@
     </row>
     <row r="23" spans="1:28" ht="29">
       <c r="A23" s="21" t="s">
-        <v>85</v>
+        <v>112</v>
       </c>
       <c r="B23" s="21" t="s">
         <v>8</v>
       </c>
       <c r="C23" s="21" t="s">
-        <v>86</v>
+        <v>113</v>
       </c>
       <c r="D23" s="21" t="s">
         <v>34</v>
@@ -3086,7 +3359,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -3101,407 +3374,433 @@
   <sheetData>
     <row r="1" spans="1:8" ht="17">
       <c r="A1" s="1" t="s">
-        <v>87</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="12" t="s">
-        <v>88</v>
+        <v>115</v>
       </c>
     </row>
     <row r="4" spans="1:8">
       <c r="A4" s="2" t="s">
-        <v>89</v>
+        <v>116</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>90</v>
+        <v>117</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>91</v>
+        <v>118</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>92</v>
+        <v>119</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>93</v>
+        <v>120</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>94</v>
+        <v>121</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>96</v>
+        <v>123</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="43.5">
       <c r="A5" s="21" t="s">
-        <v>97</v>
+        <v>124</v>
       </c>
       <c r="B5" s="21" t="s">
-        <v>98</v>
+        <v>125</v>
       </c>
       <c r="C5" s="24" t="s">
-        <v>99</v>
+        <v>126</v>
       </c>
       <c r="D5" s="21" t="s">
-        <v>100</v>
+        <v>127</v>
       </c>
       <c r="E5" s="21" t="s">
-        <v>101</v>
+        <v>128</v>
       </c>
       <c r="F5" s="21" t="s">
-        <v>102</v>
+        <v>129</v>
       </c>
       <c r="G5" s="21" t="s">
-        <v>103</v>
+        <v>130</v>
       </c>
       <c r="H5" s="21" t="s">
-        <v>104</v>
+        <v>131</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="58">
       <c r="A6" s="21" t="s">
-        <v>105</v>
+        <v>132</v>
       </c>
       <c r="B6" s="21" t="s">
-        <v>106</v>
+        <v>133</v>
       </c>
       <c r="C6" s="24" t="s">
-        <v>99</v>
+        <v>126</v>
       </c>
       <c r="D6" s="21" t="s">
-        <v>107</v>
+        <v>134</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>108</v>
+        <v>135</v>
       </c>
       <c r="F6" s="21" t="s">
-        <v>109</v>
+        <v>136</v>
       </c>
       <c r="G6" s="21" t="s">
-        <v>103</v>
+        <v>130</v>
       </c>
       <c r="H6" s="21" t="s">
-        <v>110</v>
+        <v>137</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="29">
       <c r="A7" s="21" t="s">
-        <v>111</v>
+        <v>138</v>
       </c>
       <c r="B7" s="21" t="s">
-        <v>112</v>
+        <v>139</v>
       </c>
       <c r="C7" s="24" t="s">
-        <v>99</v>
+        <v>126</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>113</v>
+        <v>140</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>114</v>
+        <v>141</v>
       </c>
       <c r="F7" s="21" t="s">
-        <v>115</v>
+        <v>142</v>
       </c>
       <c r="G7" s="21" t="s">
-        <v>116</v>
+        <v>143</v>
       </c>
       <c r="H7" s="21" t="s">
-        <v>117</v>
+        <v>144</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="29">
       <c r="A8" s="21" t="s">
-        <v>118</v>
+        <v>145</v>
       </c>
       <c r="B8" s="21" t="s">
-        <v>119</v>
+        <v>146</v>
       </c>
       <c r="C8" s="25" t="s">
-        <v>120</v>
+        <v>147</v>
       </c>
       <c r="D8" s="21" t="s">
-        <v>121</v>
+        <v>148</v>
       </c>
       <c r="E8" s="21" t="s">
-        <v>122</v>
+        <v>149</v>
       </c>
       <c r="F8" s="21" t="s">
-        <v>123</v>
+        <v>150</v>
       </c>
       <c r="G8" s="21" t="s">
-        <v>103</v>
+        <v>130</v>
       </c>
       <c r="H8" s="21" t="s">
-        <v>124</v>
+        <v>151</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="58">
       <c r="A9" s="21" t="s">
-        <v>125</v>
+        <v>152</v>
       </c>
       <c r="B9" s="21" t="s">
-        <v>126</v>
+        <v>153</v>
       </c>
       <c r="C9" s="25" t="s">
-        <v>120</v>
+        <v>147</v>
       </c>
       <c r="D9" s="21" t="s">
-        <v>127</v>
+        <v>154</v>
       </c>
       <c r="E9" s="21" t="s">
-        <v>128</v>
+        <v>155</v>
       </c>
       <c r="F9" s="21" t="s">
-        <v>129</v>
+        <v>156</v>
       </c>
       <c r="G9" s="21" t="s">
-        <v>130</v>
+        <v>157</v>
       </c>
       <c r="H9" s="21" t="s">
-        <v>131</v>
+        <v>158</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="29">
       <c r="A10" s="21" t="s">
-        <v>132</v>
+        <v>159</v>
       </c>
       <c r="B10" s="21" t="s">
-        <v>133</v>
+        <v>160</v>
       </c>
       <c r="C10" s="26" t="s">
-        <v>134</v>
+        <v>161</v>
       </c>
       <c r="D10" s="21" t="s">
-        <v>135</v>
+        <v>162</v>
       </c>
       <c r="E10" s="21" t="s">
-        <v>136</v>
+        <v>163</v>
       </c>
       <c r="F10" s="21" t="s">
-        <v>137</v>
+        <v>164</v>
       </c>
       <c r="G10" s="21" t="s">
-        <v>116</v>
+        <v>143</v>
       </c>
       <c r="H10" s="21" t="s">
-        <v>138</v>
+        <v>165</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="29">
       <c r="A11" s="21" t="s">
-        <v>139</v>
+        <v>166</v>
       </c>
       <c r="B11" s="21" t="s">
-        <v>140</v>
+        <v>167</v>
       </c>
       <c r="C11" s="24" t="s">
-        <v>99</v>
+        <v>126</v>
       </c>
       <c r="D11" s="21" t="s">
-        <v>141</v>
+        <v>168</v>
       </c>
       <c r="E11" s="21" t="s">
-        <v>142</v>
+        <v>169</v>
       </c>
       <c r="F11" s="21" t="s">
-        <v>143</v>
+        <v>170</v>
       </c>
       <c r="G11" s="21" t="s">
-        <v>103</v>
+        <v>130</v>
       </c>
       <c r="H11" s="21" t="s">
-        <v>144</v>
+        <v>171</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="43.5">
       <c r="A12" s="21" t="s">
-        <v>145</v>
+        <v>172</v>
       </c>
       <c r="B12" s="21" t="s">
-        <v>146</v>
+        <v>173</v>
       </c>
       <c r="C12" s="24" t="s">
-        <v>99</v>
+        <v>126</v>
       </c>
       <c r="D12" s="21" t="s">
-        <v>147</v>
+        <v>174</v>
       </c>
       <c r="E12" s="21" t="s">
-        <v>148</v>
+        <v>175</v>
       </c>
       <c r="F12" s="21" t="s">
-        <v>149</v>
+        <v>176</v>
       </c>
       <c r="G12" s="21" t="s">
-        <v>103</v>
+        <v>130</v>
       </c>
       <c r="H12" s="21" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="43.5">
       <c r="A13" s="21" t="s">
-        <v>151</v>
+        <v>178</v>
       </c>
       <c r="B13" s="21" t="s">
-        <v>152</v>
+        <v>179</v>
       </c>
       <c r="C13" s="25" t="s">
-        <v>120</v>
+        <v>147</v>
       </c>
       <c r="D13" s="21" t="s">
-        <v>153</v>
+        <v>180</v>
       </c>
       <c r="E13" s="21" t="s">
-        <v>154</v>
+        <v>181</v>
       </c>
       <c r="F13" s="21" t="s">
-        <v>155</v>
+        <v>182</v>
       </c>
       <c r="G13" s="21" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H13" s="21" t="s">
-        <v>157</v>
+        <v>184</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="43.5">
       <c r="A14" s="21" t="s">
-        <v>158</v>
+        <v>185</v>
       </c>
       <c r="B14" s="21" t="s">
-        <v>159</v>
+        <v>186</v>
       </c>
       <c r="C14" s="25" t="s">
-        <v>120</v>
+        <v>147</v>
       </c>
       <c r="D14" s="21" t="s">
-        <v>160</v>
+        <v>187</v>
       </c>
       <c r="E14" s="21" t="s">
-        <v>161</v>
+        <v>188</v>
       </c>
       <c r="F14" s="21" t="s">
-        <v>162</v>
+        <v>189</v>
       </c>
       <c r="G14" s="21" t="s">
-        <v>130</v>
+        <v>157</v>
       </c>
       <c r="H14" s="21" t="s">
-        <v>163</v>
+        <v>190</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="58">
       <c r="A15" s="21" t="s">
-        <v>164</v>
+        <v>191</v>
       </c>
       <c r="B15" s="21" t="s">
-        <v>165</v>
+        <v>192</v>
       </c>
       <c r="C15" s="25" t="s">
-        <v>120</v>
+        <v>147</v>
       </c>
       <c r="D15" s="21" t="s">
-        <v>166</v>
+        <v>193</v>
       </c>
       <c r="E15" s="21" t="s">
-        <v>167</v>
+        <v>194</v>
       </c>
       <c r="F15" s="21" t="s">
-        <v>168</v>
+        <v>195</v>
       </c>
       <c r="G15" s="21" t="s">
-        <v>130</v>
+        <v>157</v>
       </c>
       <c r="H15" s="21" t="s">
-        <v>169</v>
+        <v>196</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="29">
       <c r="A16" s="21" t="s">
-        <v>170</v>
+        <v>197</v>
       </c>
       <c r="B16" s="21" t="s">
-        <v>171</v>
+        <v>198</v>
       </c>
       <c r="C16" s="26" t="s">
-        <v>134</v>
+        <v>161</v>
       </c>
       <c r="D16" s="21" t="s">
-        <v>172</v>
+        <v>199</v>
       </c>
       <c r="E16" s="21" t="s">
-        <v>173</v>
+        <v>200</v>
       </c>
       <c r="F16" s="21" t="s">
-        <v>174</v>
+        <v>201</v>
       </c>
       <c r="G16" s="21" t="s">
-        <v>130</v>
+        <v>157</v>
       </c>
       <c r="H16" s="21" t="s">
-        <v>175</v>
+        <v>202</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="43.5">
       <c r="A17" s="21" t="s">
-        <v>176</v>
+        <v>203</v>
       </c>
       <c r="B17" s="21" t="s">
-        <v>177</v>
+        <v>204</v>
       </c>
       <c r="C17" s="26" t="s">
-        <v>134</v>
+        <v>161</v>
       </c>
       <c r="D17" s="21" t="s">
-        <v>178</v>
+        <v>205</v>
       </c>
       <c r="E17" s="21" t="s">
-        <v>179</v>
+        <v>206</v>
       </c>
       <c r="F17" s="21" t="s">
-        <v>180</v>
+        <v>207</v>
       </c>
       <c r="G17" s="21" t="s">
-        <v>116</v>
+        <v>143</v>
       </c>
       <c r="H17" s="21" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8">
-      <c r="A19" s="19" t="s">
-        <v>182</v>
+        <v>208</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" ht="43.5">
+      <c r="A18" s="21" t="s">
+        <v>209</v>
+      </c>
+      <c r="B18" s="21" t="s">
+        <v>210</v>
+      </c>
+      <c r="C18" s="24" t="s">
+        <v>126</v>
+      </c>
+      <c r="D18" s="21" t="s">
+        <v>211</v>
+      </c>
+      <c r="E18" s="21" t="s">
+        <v>212</v>
+      </c>
+      <c r="F18" s="21" t="s">
+        <v>213</v>
+      </c>
+      <c r="G18" s="21" t="s">
+        <v>130</v>
+      </c>
+      <c r="H18" s="21" t="s">
+        <v>214</v>
       </c>
     </row>
     <row r="20" spans="1:8">
-      <c r="B20" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="C20" s="4">
-        <f>COUNTIF($C$5:$C$17,B20)</f>
-        <v>5</v>
+      <c r="A20" s="19" t="s">
+        <v>215</v>
       </c>
     </row>
     <row r="21" spans="1:8">
       <c r="B21" s="4" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="C21" s="4">
-        <f>COUNTIF($C$5:$C$17,B21)</f>
-        <v>5</v>
+        <f>COUNTIF($C$5:$C$18,B21)</f>
+        <v>6</v>
       </c>
     </row>
     <row r="22" spans="1:8">
       <c r="B22" s="4" t="s">
-        <v>134</v>
+        <v>147</v>
       </c>
       <c r="C22" s="4">
-        <f>COUNTIF($C$5:$C$17,B22)</f>
+        <f>COUNTIF($C$5:$C$18,B22)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8">
+      <c r="B23" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="C23" s="4">
+        <f>COUNTIF($C$5:$C$18,B23)</f>
         <v>3</v>
       </c>
     </row>
@@ -3520,42 +3819,42 @@
   <sheetData>
     <row r="1" spans="1:1" ht="15.5">
       <c r="A1" s="27" t="s">
-        <v>183</v>
+        <v>216</v>
       </c>
     </row>
     <row r="3" spans="1:1" ht="29">
       <c r="A3" s="28" t="s">
-        <v>184</v>
+        <v>217</v>
       </c>
     </row>
     <row r="4" spans="1:1" ht="29">
       <c r="A4" s="28" t="s">
-        <v>185</v>
+        <v>218</v>
       </c>
     </row>
     <row r="5" spans="1:1" ht="29">
       <c r="A5" s="28" t="s">
-        <v>186</v>
+        <v>219</v>
       </c>
     </row>
     <row r="6" spans="1:1" ht="29">
       <c r="A6" s="28" t="s">
-        <v>187</v>
+        <v>220</v>
       </c>
     </row>
     <row r="7" spans="1:1" ht="29">
       <c r="A7" s="28" t="s">
-        <v>188</v>
+        <v>221</v>
       </c>
     </row>
     <row r="8" spans="1:1">
       <c r="A8" s="28" t="s">
-        <v>189</v>
+        <v>222</v>
       </c>
     </row>
     <row r="9" spans="1:1">
       <c r="A9" s="28" t="s">
-        <v>190</v>
+        <v>223</v>
       </c>
     </row>
   </sheetData>

</xml_diff>